<commit_message>
Logistic Regression Tutorial (Multiclass Classification)
</commit_message>
<xml_diff>
--- a/ML/2) Supervise Machine Learning Classification/ML_Classification_PrecisionRecall_resources/precision_recall.xlsx
+++ b/ML/2) Supervise Machine Learning Classification/ML_Classification_PrecisionRecall_resources/precision_recall.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ML\ch2_supervised_learning_classification\2_precision_recall\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\ML\2) Supervise Machine Learning Classification\ML_Classification_PrecisionRecall_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26CBE1EF-1F71-4ABD-A36F-AF6407173F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E005F96D-8963-4A5F-80D3-B7C21CC24543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10620" yWindow="0" windowWidth="12516" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Recall</t>
   </si>
@@ -54,6 +52,9 @@
   </si>
   <si>
     <t>truth (y_test)</t>
+  </si>
+  <si>
+    <t>F1 Score</t>
   </si>
 </sst>
 </file>
@@ -394,19 +395,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="23.4" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="21.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="31.5703125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="27.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.21875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -419,8 +421,11 @@
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -438,8 +443,12 @@
         <f>5/5</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G2" s="1">
+        <f>2*(E2*F2)/(E2+F2)</f>
+        <v>0.90909090909090906</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -457,8 +466,12 @@
         <f>3/4</f>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G3" s="1">
+        <f>2*E3*F3/(E3+F3)</f>
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -466,7 +479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>0</v>
       </c>
@@ -474,7 +487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>0</v>
       </c>
@@ -482,7 +495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>0</v>
       </c>
@@ -490,7 +503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -498,7 +511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -506,7 +519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>0</v>
       </c>

</xml_diff>